<commit_message>
feat: update import for switch, ap, proyector
</commit_message>
<xml_diff>
--- a/public/formato_importar_activo.xlsx
+++ b/public/formato_importar_activo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Estudiante\Desktop\Inventario FCSH\Código\Front y Back\frontend-fcsh\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56E7EB93-7186-49B4-92D2-2DAB63E203B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0622AB3-0072-4240-A941-3D20D48FD0C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{2D0AE001-BFB5-4376-BAB2-74157DEC9722}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{2D0AE001-BFB5-4376-BAB2-74157DEC9722}"/>
   </bookViews>
   <sheets>
     <sheet name="Computadora" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="49">
   <si>
     <t>Id</t>
   </si>
@@ -175,9 +175,6 @@
   </si>
   <si>
     <t>Nombre</t>
-  </si>
-  <si>
-    <t>Empresa</t>
   </si>
   <si>
     <t>N°</t>
@@ -293,38 +290,9 @@
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -333,7 +301,6 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -342,67 +309,15 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -411,12 +326,91 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
         </patternFill>
       </fill>
     </dxf>
@@ -559,14 +553,6 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color indexed="64"/>
@@ -698,14 +684,6 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color indexed="64"/>
@@ -825,6 +803,25 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <border outline="0">
@@ -876,36 +873,36 @@
     <tableColumn id="1" xr3:uid="{69EE392B-C8B4-40F4-8A09-D5B4BBB77C93}" name="Id"/>
     <tableColumn id="2" xr3:uid="{5A3CDC4A-1650-4A0F-B9F7-CC6FAC7BDB28}" name="Edificio"/>
     <tableColumn id="3" xr3:uid="{570F8650-9BD3-4952-BAFF-35E1BD8DBBCE}" name="No. Aula"/>
-    <tableColumn id="4" xr3:uid="{80117818-1838-4A8D-8961-70420F30C222}" name="Oficina" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{77BA4D51-6F62-4751-971C-0EE4A7FD727C}" name="Usuario" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{23869ECA-ED25-4414-832A-F62341274D5D}" name="Uso" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{2624E368-C572-4558-B277-40C78CC4FBE9}" name="Tipo" dataDxfId="79"/>
-    <tableColumn id="35" xr3:uid="{262F381F-F127-425F-BAE3-183AAC930981}" name="Año Adq" dataDxfId="78"/>
-    <tableColumn id="8" xr3:uid="{B5D02DC1-FF2D-43B9-B6C4-237415A70E29}" name="IP" dataDxfId="77"/>
-    <tableColumn id="10" xr3:uid="{02832541-384B-401D-9FB1-324B032E95D2}" name="Nombre de equipo" dataDxfId="76"/>
-    <tableColumn id="11" xr3:uid="{C676392C-E1C8-4A0F-9BB8-73B0714052C4}" name="Dominio" dataDxfId="75"/>
-    <tableColumn id="12" xr3:uid="{7212E756-C5D1-4E56-A2D5-A966E7461136}" name="Sistema Operativo" dataDxfId="74"/>
-    <tableColumn id="34" xr3:uid="{1D11890E-D69E-47C1-B1D5-35D26F7E9493}" name="Versión" dataDxfId="73"/>
-    <tableColumn id="13" xr3:uid="{7C63AAE4-FC27-49E8-8CDF-F5AB4C3F4203}" name="Procesador" dataDxfId="72"/>
-    <tableColumn id="14" xr3:uid="{874D42EB-6761-4C40-BA8C-D630F5CAF141}" name="Capacidad Memoria" dataDxfId="71"/>
-    <tableColumn id="15" xr3:uid="{A074245F-4DE0-43CC-929D-12D5AB3A6F06}" name="Capacidad HDD" dataDxfId="70"/>
-    <tableColumn id="36" xr3:uid="{3FF7C9C2-C228-4BAD-9A2D-C891BA443C49}" name="Tipo Disco" dataDxfId="69"/>
-    <tableColumn id="16" xr3:uid="{21C45942-9F0B-4731-B63B-258BE1A47F68}" name="Marca Case" dataDxfId="68"/>
-    <tableColumn id="17" xr3:uid="{0B1A272A-CF22-4B2B-8C4A-FF26F85A236C}" name="Modelo Case" dataDxfId="67"/>
-    <tableColumn id="18" xr3:uid="{FD33D26C-399A-4ED9-AFFE-174C7F55071D}" name="Serie CPU" dataDxfId="66"/>
-    <tableColumn id="19" xr3:uid="{7D4D2208-3CD9-4E17-8260-B44A49F5652C}" name="Marca monitor" dataDxfId="65"/>
-    <tableColumn id="20" xr3:uid="{D8DA6A4A-F618-4B5C-99FC-B3CA92E8841E}" name="Modelo monitor" dataDxfId="64"/>
-    <tableColumn id="21" xr3:uid="{E8DC5050-5DFC-43F2-9FEF-72E5F0A201B5}" name="Serie monitor" dataDxfId="63"/>
-    <tableColumn id="22" xr3:uid="{B111462E-807B-459E-9EAF-889D59FC3370}" name="Marca teclado" dataDxfId="62"/>
-    <tableColumn id="23" xr3:uid="{D909F966-7AD4-4A8C-950D-259B356F2C1D}" name="Modelo teclado" dataDxfId="61"/>
-    <tableColumn id="24" xr3:uid="{20E9A183-CB25-4C40-8556-9A7B4DE433C2}" name="Serie teclado" dataDxfId="60"/>
-    <tableColumn id="25" xr3:uid="{67ACBD13-24EF-47FB-99C0-D33EAE32794D}" name="Marca mouse" dataDxfId="59"/>
-    <tableColumn id="26" xr3:uid="{FC104ADA-C3DD-4872-9134-A8F359CD92ED}" name="Modelo mouse" dataDxfId="58"/>
-    <tableColumn id="27" xr3:uid="{72913F84-BFE6-4F18-B568-78A034CF91E0}" name="Serie mouse" dataDxfId="57"/>
-    <tableColumn id="28" xr3:uid="{9503ECC5-F543-47DD-B05F-BE5CFED614E7}" name="Inventario CPU" dataDxfId="56"/>
-    <tableColumn id="29" xr3:uid="{F23D81CF-45FF-4B42-AE1D-C3FF20A02D47}" name="Inventario Monitor" dataDxfId="55"/>
-    <tableColumn id="30" xr3:uid="{5E7F41A6-23EE-49FF-B9A7-67B41746BA02}" name="Inventario Teclado" dataDxfId="54"/>
-    <tableColumn id="31" xr3:uid="{E73A3977-4E78-4BBD-B43C-5CDDDFB5A0B5}" name="Inventario Mouse" dataDxfId="53"/>
+    <tableColumn id="4" xr3:uid="{80117818-1838-4A8D-8961-70420F30C222}" name="Oficina" dataDxfId="79"/>
+    <tableColumn id="5" xr3:uid="{77BA4D51-6F62-4751-971C-0EE4A7FD727C}" name="Usuario" dataDxfId="78"/>
+    <tableColumn id="6" xr3:uid="{23869ECA-ED25-4414-832A-F62341274D5D}" name="Uso" dataDxfId="77"/>
+    <tableColumn id="7" xr3:uid="{2624E368-C572-4558-B277-40C78CC4FBE9}" name="Tipo" dataDxfId="76"/>
+    <tableColumn id="35" xr3:uid="{262F381F-F127-425F-BAE3-183AAC930981}" name="Año Adq" dataDxfId="75"/>
+    <tableColumn id="8" xr3:uid="{B5D02DC1-FF2D-43B9-B6C4-237415A70E29}" name="IP" dataDxfId="74"/>
+    <tableColumn id="10" xr3:uid="{02832541-384B-401D-9FB1-324B032E95D2}" name="Nombre de equipo" dataDxfId="73"/>
+    <tableColumn id="11" xr3:uid="{C676392C-E1C8-4A0F-9BB8-73B0714052C4}" name="Dominio" dataDxfId="72"/>
+    <tableColumn id="12" xr3:uid="{7212E756-C5D1-4E56-A2D5-A966E7461136}" name="Sistema Operativo" dataDxfId="71"/>
+    <tableColumn id="34" xr3:uid="{1D11890E-D69E-47C1-B1D5-35D26F7E9493}" name="Versión" dataDxfId="70"/>
+    <tableColumn id="13" xr3:uid="{7C63AAE4-FC27-49E8-8CDF-F5AB4C3F4203}" name="Procesador" dataDxfId="69"/>
+    <tableColumn id="14" xr3:uid="{874D42EB-6761-4C40-BA8C-D630F5CAF141}" name="Capacidad Memoria" dataDxfId="68"/>
+    <tableColumn id="15" xr3:uid="{A074245F-4DE0-43CC-929D-12D5AB3A6F06}" name="Capacidad HDD" dataDxfId="67"/>
+    <tableColumn id="36" xr3:uid="{3FF7C9C2-C228-4BAD-9A2D-C891BA443C49}" name="Tipo Disco" dataDxfId="66"/>
+    <tableColumn id="16" xr3:uid="{21C45942-9F0B-4731-B63B-258BE1A47F68}" name="Marca Case" dataDxfId="65"/>
+    <tableColumn id="17" xr3:uid="{0B1A272A-CF22-4B2B-8C4A-FF26F85A236C}" name="Modelo Case" dataDxfId="64"/>
+    <tableColumn id="18" xr3:uid="{FD33D26C-399A-4ED9-AFFE-174C7F55071D}" name="Serie CPU" dataDxfId="63"/>
+    <tableColumn id="19" xr3:uid="{7D4D2208-3CD9-4E17-8260-B44A49F5652C}" name="Marca monitor" dataDxfId="62"/>
+    <tableColumn id="20" xr3:uid="{D8DA6A4A-F618-4B5C-99FC-B3CA92E8841E}" name="Modelo monitor" dataDxfId="61"/>
+    <tableColumn id="21" xr3:uid="{E8DC5050-5DFC-43F2-9FEF-72E5F0A201B5}" name="Serie monitor" dataDxfId="60"/>
+    <tableColumn id="22" xr3:uid="{B111462E-807B-459E-9EAF-889D59FC3370}" name="Marca teclado" dataDxfId="59"/>
+    <tableColumn id="23" xr3:uid="{D909F966-7AD4-4A8C-950D-259B356F2C1D}" name="Modelo teclado" dataDxfId="58"/>
+    <tableColumn id="24" xr3:uid="{20E9A183-CB25-4C40-8556-9A7B4DE433C2}" name="Serie teclado" dataDxfId="57"/>
+    <tableColumn id="25" xr3:uid="{67ACBD13-24EF-47FB-99C0-D33EAE32794D}" name="Marca mouse" dataDxfId="56"/>
+    <tableColumn id="26" xr3:uid="{FC104ADA-C3DD-4872-9134-A8F359CD92ED}" name="Modelo mouse" dataDxfId="55"/>
+    <tableColumn id="27" xr3:uid="{72913F84-BFE6-4F18-B568-78A034CF91E0}" name="Serie mouse" dataDxfId="54"/>
+    <tableColumn id="28" xr3:uid="{9503ECC5-F543-47DD-B05F-BE5CFED614E7}" name="Inventario CPU" dataDxfId="53"/>
+    <tableColumn id="29" xr3:uid="{F23D81CF-45FF-4B42-AE1D-C3FF20A02D47}" name="Inventario Monitor" dataDxfId="52"/>
+    <tableColumn id="30" xr3:uid="{5E7F41A6-23EE-49FF-B9A7-67B41746BA02}" name="Inventario Teclado" dataDxfId="51"/>
+    <tableColumn id="31" xr3:uid="{E73A3977-4E78-4BBD-B43C-5CDDDFB5A0B5}" name="Inventario Mouse" dataDxfId="50"/>
     <tableColumn id="32" xr3:uid="{132BAE04-41F0-4D14-886F-EE4B5E17AA48}" name="Observación"/>
     <tableColumn id="33" xr3:uid="{75F5651F-591E-4487-8692-3B6B587F55ED}" name="Fecha si se hace cambio"/>
   </tableColumns>
@@ -914,53 +911,53 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{65571BBC-6721-44F4-B921-CE5855D2DD45}" name="Tabla13" displayName="Tabla13" ref="A1:L2" insertRow="1" totalsRowShown="0" headerRowDxfId="52" dataDxfId="50" headerRowBorderDxfId="51" tableBorderDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{65571BBC-6721-44F4-B921-CE5855D2DD45}" name="Tabla13" displayName="Tabla13" ref="A1:L2" insertRow="1" totalsRowShown="0" headerRowDxfId="49" dataDxfId="47" headerRowBorderDxfId="48" tableBorderDxfId="46">
   <autoFilter ref="A1:L2" xr:uid="{65571BBC-6721-44F4-B921-CE5855D2DD45}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{FDE9EEEE-D60D-45CB-A800-B53803E8A3B8}" name="N°" dataDxfId="48"/>
-    <tableColumn id="2" xr3:uid="{DEE49521-B61A-4DCE-BA47-2362448B1284}" name="Empresa" dataDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{1B2D9558-F9ED-4CCE-9E02-C266643535C2}" name="Inventario" dataDxfId="46"/>
-    <tableColumn id="4" xr3:uid="{F9374C12-7D10-4F8D-A9F2-6B74A4324A16}" name="Bloque" dataDxfId="45"/>
-    <tableColumn id="5" xr3:uid="{CC47AE73-F008-4779-8A1E-999613B73F36}" name="Ubicación" dataDxfId="44"/>
-    <tableColumn id="6" xr3:uid="{C4B7087C-C5A9-418F-973B-91019B7B4D85}" name="Marca" dataDxfId="43"/>
-    <tableColumn id="7" xr3:uid="{A29FE592-5D13-4856-A8B2-D3757F7FE5D1}" name="Modelo" dataDxfId="42"/>
-    <tableColumn id="35" xr3:uid="{28CE02F8-C218-4318-91D6-3221A4C1677C}" name="Serie" dataDxfId="41"/>
-    <tableColumn id="8" xr3:uid="{D6339E67-64E9-4609-AE94-03511A1E2DFA}" name="Categoría" dataDxfId="40"/>
-    <tableColumn id="10" xr3:uid="{BC81D9A6-A156-4735-B029-2F2D63CB0EBE}" name="Lámpara" dataDxfId="39"/>
-    <tableColumn id="11" xr3:uid="{EC220C64-81F8-4715-812E-830F143FAFE1}" name="Estado" dataDxfId="38"/>
-    <tableColumn id="12" xr3:uid="{520BC8C9-05B0-4EE0-A833-D9F61A0DD0AB}" name="Observación" dataDxfId="37"/>
+    <tableColumn id="1" xr3:uid="{FDE9EEEE-D60D-45CB-A800-B53803E8A3B8}" name="N°" dataDxfId="45"/>
+    <tableColumn id="9" xr3:uid="{0F2C1BC4-B276-43C3-8519-94D5DE11E4D7}" name="Año Adq" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{1B2D9558-F9ED-4CCE-9E02-C266643535C2}" name="Inventario" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{F9374C12-7D10-4F8D-A9F2-6B74A4324A16}" name="Bloque" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{CC47AE73-F008-4779-8A1E-999613B73F36}" name="Ubicación" dataDxfId="42"/>
+    <tableColumn id="6" xr3:uid="{C4B7087C-C5A9-418F-973B-91019B7B4D85}" name="Marca" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{A29FE592-5D13-4856-A8B2-D3757F7FE5D1}" name="Modelo" dataDxfId="40"/>
+    <tableColumn id="35" xr3:uid="{28CE02F8-C218-4318-91D6-3221A4C1677C}" name="Serie" dataDxfId="39"/>
+    <tableColumn id="8" xr3:uid="{D6339E67-64E9-4609-AE94-03511A1E2DFA}" name="Categoría" dataDxfId="38"/>
+    <tableColumn id="10" xr3:uid="{BC81D9A6-A156-4735-B029-2F2D63CB0EBE}" name="Lámpara" dataDxfId="37"/>
+    <tableColumn id="11" xr3:uid="{EC220C64-81F8-4715-812E-830F143FAFE1}" name="Estado" dataDxfId="36"/>
+    <tableColumn id="12" xr3:uid="{520BC8C9-05B0-4EE0-A833-D9F61A0DD0AB}" name="Observación" dataDxfId="35"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{117726C3-B927-45D2-BCB6-906E81362D65}" name="Tabla134" displayName="Tabla134" ref="A1:L2" insertRow="1" totalsRowShown="0" headerRowDxfId="36" dataDxfId="34" headerRowBorderDxfId="35" tableBorderDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{117726C3-B927-45D2-BCB6-906E81362D65}" name="Tabla134" displayName="Tabla134" ref="A1:L2" insertRow="1" totalsRowShown="0" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33" tableBorderDxfId="31">
   <autoFilter ref="A1:L2" xr:uid="{117726C3-B927-45D2-BCB6-906E81362D65}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{276C8004-7E62-4A99-99B6-54C1CCAB9A0D}" name="N°" dataDxfId="32"/>
-    <tableColumn id="2" xr3:uid="{C9F3FDD4-4F0A-4DA9-AF0B-5EB36C832A27}" name="Empresa" dataDxfId="31"/>
-    <tableColumn id="59" xr3:uid="{2EDF8951-57A8-4DA8-83DD-41E4ABB04F28}" name="Nombre" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{6C6FAF5E-4416-4701-AF7F-C6B09875F0E3}" name="Inventario" dataDxfId="29"/>
-    <tableColumn id="4" xr3:uid="{9009A994-0659-4EB2-A948-BB850B7E7869}" name="Bloque" dataDxfId="28"/>
-    <tableColumn id="5" xr3:uid="{2BFE8A4C-F74C-4478-94F2-9CDCD7517FF5}" name="Ubicación" dataDxfId="27"/>
-    <tableColumn id="6" xr3:uid="{C3F80FC4-FC88-4067-86B5-9E0F39992776}" name="Marca" dataDxfId="26"/>
-    <tableColumn id="7" xr3:uid="{1EB67BDD-CF6B-448D-A8ED-A99A60F26085}" name="Modelo" dataDxfId="25"/>
-    <tableColumn id="35" xr3:uid="{4F1E28EC-460F-4A15-A541-75DDC5A3B10F}" name="Serie" dataDxfId="24"/>
-    <tableColumn id="11" xr3:uid="{646DF198-108C-4FD8-BA3F-221C547C787D}" name="MAC" dataDxfId="23"/>
-    <tableColumn id="61" xr3:uid="{0F76C99C-FD25-4F18-AC82-BC0A9BD0BFC3}" name="Estado" dataDxfId="22"/>
-    <tableColumn id="12" xr3:uid="{DA153594-3249-41ED-9088-5D447B2330F5}" name="Observación" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{276C8004-7E62-4A99-99B6-54C1CCAB9A0D}" name="N°" dataDxfId="30"/>
+    <tableColumn id="8" xr3:uid="{5DC544D0-D6BC-4180-8835-12C885A89DB4}" name="Año Adq" dataDxfId="1"/>
+    <tableColumn id="59" xr3:uid="{2EDF8951-57A8-4DA8-83DD-41E4ABB04F28}" name="Nombre" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{6C6FAF5E-4416-4701-AF7F-C6B09875F0E3}" name="Inventario" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{9009A994-0659-4EB2-A948-BB850B7E7869}" name="Bloque" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{2BFE8A4C-F74C-4478-94F2-9CDCD7517FF5}" name="Ubicación" dataDxfId="26"/>
+    <tableColumn id="6" xr3:uid="{C3F80FC4-FC88-4067-86B5-9E0F39992776}" name="Marca" dataDxfId="25"/>
+    <tableColumn id="7" xr3:uid="{1EB67BDD-CF6B-448D-A8ED-A99A60F26085}" name="Modelo" dataDxfId="24"/>
+    <tableColumn id="35" xr3:uid="{4F1E28EC-460F-4A15-A541-75DDC5A3B10F}" name="Serie" dataDxfId="23"/>
+    <tableColumn id="11" xr3:uid="{646DF198-108C-4FD8-BA3F-221C547C787D}" name="MAC" dataDxfId="22"/>
+    <tableColumn id="61" xr3:uid="{0F76C99C-FD25-4F18-AC82-BC0A9BD0BFC3}" name="Estado" dataDxfId="21"/>
+    <tableColumn id="12" xr3:uid="{DA153594-3249-41ED-9088-5D447B2330F5}" name="Observación" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{81C6E5BE-3A2E-49E1-B3C1-BD159715F86B}" name="Tabla1345" displayName="Tabla1345" ref="A1:N2" insertRow="1" totalsRowShown="0" headerRowDxfId="20" dataDxfId="18" headerRowBorderDxfId="19" tableBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{81C6E5BE-3A2E-49E1-B3C1-BD159715F86B}" name="Tabla1345" displayName="Tabla1345" ref="A1:N2" insertRow="1" totalsRowShown="0" headerRowDxfId="19" dataDxfId="17" headerRowBorderDxfId="18" tableBorderDxfId="16">
   <autoFilter ref="A1:N2" xr:uid="{81C6E5BE-3A2E-49E1-B3C1-BD159715F86B}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{5752E7FC-405F-447F-B9C8-E1DD962FB1D1}" name="N°" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{5D7757C9-37E0-45A7-ADC0-4F94CECEB175}" name="Empresa" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{5752E7FC-405F-447F-B9C8-E1DD962FB1D1}" name="N°" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{8DECD9A9-F47F-4F5A-B630-9B1F78EDD65B}" name="Año Adq" dataDxfId="0"/>
     <tableColumn id="59" xr3:uid="{6E508FCA-0F19-4A5A-97A2-4220449D6882}" name="Nombre" dataDxfId="14"/>
     <tableColumn id="3" xr3:uid="{F0B5BEAE-2A98-4302-9893-9D181D3E666D}" name="Inventario" dataDxfId="13"/>
     <tableColumn id="4" xr3:uid="{1F479286-0DEA-4626-AB22-A4F8CC3FE875}" name="Bloque" dataDxfId="12"/>
@@ -1454,10 +1451,10 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>42</v>
@@ -1478,10 +1475,10 @@
         <v>37</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>36</v>
@@ -1520,10 +1517,10 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>43</v>
@@ -1585,10 +1582,10 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>43</v>
@@ -1615,10 +1612,10 @@
         <v>33</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
feat: update import format
</commit_message>
<xml_diff>
--- a/public/formato_importar_activo.xlsx
+++ b/public/formato_importar_activo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Estudiante\Desktop\Inventario FCSH\Código\Front y Back\frontend-fcsh\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0622AB3-0072-4240-A941-3D20D48FD0C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0A9DD25-40F4-495E-A803-F0FACF6934AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{2D0AE001-BFB5-4376-BAB2-74157DEC9722}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{2D0AE001-BFB5-4376-BAB2-74157DEC9722}"/>
   </bookViews>
   <sheets>
     <sheet name="Computadora" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="49">
   <si>
     <t>Id</t>
   </si>
@@ -141,9 +141,6 @@
     <t>Observación</t>
   </si>
   <si>
-    <t>Fecha si se hace cambio</t>
-  </si>
-  <si>
     <t>MAC</t>
   </si>
   <si>
@@ -190,6 +187,9 @@
   </si>
   <si>
     <t>Categoría</t>
+  </si>
+  <si>
+    <t>Empresa</t>
   </si>
 </sst>
 </file>
@@ -257,7 +257,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -280,12 +280,22 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{C683BCB6-F98D-4AB2-84B8-29BDC748D3E0}"/>
   </cellStyles>
-  <dxfs count="84">
+  <dxfs count="88">
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="none">
@@ -293,6 +303,7 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -301,6 +312,7 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -309,15 +321,67 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -326,83 +390,12 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
           <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -548,6 +541,22 @@
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
           <bgColor auto="1"/>
         </patternFill>
       </fill>
@@ -679,6 +688,22 @@
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
           <bgColor auto="1"/>
         </patternFill>
       </fill>
@@ -763,6 +788,9 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -867,109 +895,112 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A20B7714-7766-4C9C-B6E9-104829CF83F7}" name="Tabla1" displayName="Tabla1" ref="A1:AI2" insertRow="1" totalsRowShown="0" headerRowDxfId="83" dataDxfId="81" headerRowBorderDxfId="82" tableBorderDxfId="80">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A20B7714-7766-4C9C-B6E9-104829CF83F7}" name="Tabla1" displayName="Tabla1" ref="A1:AI2" insertRow="1" totalsRowShown="0" headerRowDxfId="87" dataDxfId="85" headerRowBorderDxfId="86" tableBorderDxfId="84">
   <autoFilter ref="A1:AI2" xr:uid="{527E07F6-196F-429B-AB65-4AB51DC1A29B}"/>
   <tableColumns count="35">
     <tableColumn id="1" xr3:uid="{69EE392B-C8B4-40F4-8A09-D5B4BBB77C93}" name="Id"/>
     <tableColumn id="2" xr3:uid="{5A3CDC4A-1650-4A0F-B9F7-CC6FAC7BDB28}" name="Edificio"/>
     <tableColumn id="3" xr3:uid="{570F8650-9BD3-4952-BAFF-35E1BD8DBBCE}" name="No. Aula"/>
-    <tableColumn id="4" xr3:uid="{80117818-1838-4A8D-8961-70420F30C222}" name="Oficina" dataDxfId="79"/>
-    <tableColumn id="5" xr3:uid="{77BA4D51-6F62-4751-971C-0EE4A7FD727C}" name="Usuario" dataDxfId="78"/>
-    <tableColumn id="6" xr3:uid="{23869ECA-ED25-4414-832A-F62341274D5D}" name="Uso" dataDxfId="77"/>
-    <tableColumn id="7" xr3:uid="{2624E368-C572-4558-B277-40C78CC4FBE9}" name="Tipo" dataDxfId="76"/>
-    <tableColumn id="35" xr3:uid="{262F381F-F127-425F-BAE3-183AAC930981}" name="Año Adq" dataDxfId="75"/>
-    <tableColumn id="8" xr3:uid="{B5D02DC1-FF2D-43B9-B6C4-237415A70E29}" name="IP" dataDxfId="74"/>
-    <tableColumn id="10" xr3:uid="{02832541-384B-401D-9FB1-324B032E95D2}" name="Nombre de equipo" dataDxfId="73"/>
-    <tableColumn id="11" xr3:uid="{C676392C-E1C8-4A0F-9BB8-73B0714052C4}" name="Dominio" dataDxfId="72"/>
-    <tableColumn id="12" xr3:uid="{7212E756-C5D1-4E56-A2D5-A966E7461136}" name="Sistema Operativo" dataDxfId="71"/>
-    <tableColumn id="34" xr3:uid="{1D11890E-D69E-47C1-B1D5-35D26F7E9493}" name="Versión" dataDxfId="70"/>
-    <tableColumn id="13" xr3:uid="{7C63AAE4-FC27-49E8-8CDF-F5AB4C3F4203}" name="Procesador" dataDxfId="69"/>
-    <tableColumn id="14" xr3:uid="{874D42EB-6761-4C40-BA8C-D630F5CAF141}" name="Capacidad Memoria" dataDxfId="68"/>
-    <tableColumn id="15" xr3:uid="{A074245F-4DE0-43CC-929D-12D5AB3A6F06}" name="Capacidad HDD" dataDxfId="67"/>
-    <tableColumn id="36" xr3:uid="{3FF7C9C2-C228-4BAD-9A2D-C891BA443C49}" name="Tipo Disco" dataDxfId="66"/>
-    <tableColumn id="16" xr3:uid="{21C45942-9F0B-4731-B63B-258BE1A47F68}" name="Marca Case" dataDxfId="65"/>
-    <tableColumn id="17" xr3:uid="{0B1A272A-CF22-4B2B-8C4A-FF26F85A236C}" name="Modelo Case" dataDxfId="64"/>
-    <tableColumn id="18" xr3:uid="{FD33D26C-399A-4ED9-AFFE-174C7F55071D}" name="Serie CPU" dataDxfId="63"/>
-    <tableColumn id="19" xr3:uid="{7D4D2208-3CD9-4E17-8260-B44A49F5652C}" name="Marca monitor" dataDxfId="62"/>
-    <tableColumn id="20" xr3:uid="{D8DA6A4A-F618-4B5C-99FC-B3CA92E8841E}" name="Modelo monitor" dataDxfId="61"/>
-    <tableColumn id="21" xr3:uid="{E8DC5050-5DFC-43F2-9FEF-72E5F0A201B5}" name="Serie monitor" dataDxfId="60"/>
-    <tableColumn id="22" xr3:uid="{B111462E-807B-459E-9EAF-889D59FC3370}" name="Marca teclado" dataDxfId="59"/>
-    <tableColumn id="23" xr3:uid="{D909F966-7AD4-4A8C-950D-259B356F2C1D}" name="Modelo teclado" dataDxfId="58"/>
-    <tableColumn id="24" xr3:uid="{20E9A183-CB25-4C40-8556-9A7B4DE433C2}" name="Serie teclado" dataDxfId="57"/>
-    <tableColumn id="25" xr3:uid="{67ACBD13-24EF-47FB-99C0-D33EAE32794D}" name="Marca mouse" dataDxfId="56"/>
-    <tableColumn id="26" xr3:uid="{FC104ADA-C3DD-4872-9134-A8F359CD92ED}" name="Modelo mouse" dataDxfId="55"/>
-    <tableColumn id="27" xr3:uid="{72913F84-BFE6-4F18-B568-78A034CF91E0}" name="Serie mouse" dataDxfId="54"/>
-    <tableColumn id="28" xr3:uid="{9503ECC5-F543-47DD-B05F-BE5CFED614E7}" name="Inventario CPU" dataDxfId="53"/>
-    <tableColumn id="29" xr3:uid="{F23D81CF-45FF-4B42-AE1D-C3FF20A02D47}" name="Inventario Monitor" dataDxfId="52"/>
-    <tableColumn id="30" xr3:uid="{5E7F41A6-23EE-49FF-B9A7-67B41746BA02}" name="Inventario Teclado" dataDxfId="51"/>
-    <tableColumn id="31" xr3:uid="{E73A3977-4E78-4BBD-B43C-5CDDDFB5A0B5}" name="Inventario Mouse" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{80117818-1838-4A8D-8961-70420F30C222}" name="Oficina" dataDxfId="83"/>
+    <tableColumn id="5" xr3:uid="{77BA4D51-6F62-4751-971C-0EE4A7FD727C}" name="Usuario" dataDxfId="82"/>
+    <tableColumn id="6" xr3:uid="{23869ECA-ED25-4414-832A-F62341274D5D}" name="Uso" dataDxfId="81"/>
+    <tableColumn id="7" xr3:uid="{2624E368-C572-4558-B277-40C78CC4FBE9}" name="Tipo" dataDxfId="80"/>
+    <tableColumn id="9" xr3:uid="{81C7EE1F-BD27-4C04-BFAC-386377E200AF}" name="Empresa" dataDxfId="79"/>
+    <tableColumn id="35" xr3:uid="{262F381F-F127-425F-BAE3-183AAC930981}" name="Año Adq" dataDxfId="78"/>
+    <tableColumn id="8" xr3:uid="{B5D02DC1-FF2D-43B9-B6C4-237415A70E29}" name="IP" dataDxfId="77"/>
+    <tableColumn id="10" xr3:uid="{02832541-384B-401D-9FB1-324B032E95D2}" name="Nombre de equipo" dataDxfId="76"/>
+    <tableColumn id="11" xr3:uid="{C676392C-E1C8-4A0F-9BB8-73B0714052C4}" name="Dominio" dataDxfId="75"/>
+    <tableColumn id="12" xr3:uid="{7212E756-C5D1-4E56-A2D5-A966E7461136}" name="Sistema Operativo" dataDxfId="74"/>
+    <tableColumn id="34" xr3:uid="{1D11890E-D69E-47C1-B1D5-35D26F7E9493}" name="Versión" dataDxfId="73"/>
+    <tableColumn id="13" xr3:uid="{7C63AAE4-FC27-49E8-8CDF-F5AB4C3F4203}" name="Procesador" dataDxfId="72"/>
+    <tableColumn id="14" xr3:uid="{874D42EB-6761-4C40-BA8C-D630F5CAF141}" name="Capacidad Memoria" dataDxfId="71"/>
+    <tableColumn id="15" xr3:uid="{A074245F-4DE0-43CC-929D-12D5AB3A6F06}" name="Capacidad HDD" dataDxfId="70"/>
+    <tableColumn id="36" xr3:uid="{3FF7C9C2-C228-4BAD-9A2D-C891BA443C49}" name="Tipo Disco" dataDxfId="69"/>
+    <tableColumn id="16" xr3:uid="{21C45942-9F0B-4731-B63B-258BE1A47F68}" name="Marca Case" dataDxfId="68"/>
+    <tableColumn id="17" xr3:uid="{0B1A272A-CF22-4B2B-8C4A-FF26F85A236C}" name="Modelo Case" dataDxfId="67"/>
+    <tableColumn id="18" xr3:uid="{FD33D26C-399A-4ED9-AFFE-174C7F55071D}" name="Serie CPU" dataDxfId="66"/>
+    <tableColumn id="19" xr3:uid="{7D4D2208-3CD9-4E17-8260-B44A49F5652C}" name="Marca monitor" dataDxfId="65"/>
+    <tableColumn id="20" xr3:uid="{D8DA6A4A-F618-4B5C-99FC-B3CA92E8841E}" name="Modelo monitor" dataDxfId="64"/>
+    <tableColumn id="21" xr3:uid="{E8DC5050-5DFC-43F2-9FEF-72E5F0A201B5}" name="Serie monitor" dataDxfId="63"/>
+    <tableColumn id="22" xr3:uid="{B111462E-807B-459E-9EAF-889D59FC3370}" name="Marca teclado" dataDxfId="62"/>
+    <tableColumn id="23" xr3:uid="{D909F966-7AD4-4A8C-950D-259B356F2C1D}" name="Modelo teclado" dataDxfId="61"/>
+    <tableColumn id="24" xr3:uid="{20E9A183-CB25-4C40-8556-9A7B4DE433C2}" name="Serie teclado" dataDxfId="60"/>
+    <tableColumn id="25" xr3:uid="{67ACBD13-24EF-47FB-99C0-D33EAE32794D}" name="Marca mouse" dataDxfId="59"/>
+    <tableColumn id="26" xr3:uid="{FC104ADA-C3DD-4872-9134-A8F359CD92ED}" name="Modelo mouse" dataDxfId="58"/>
+    <tableColumn id="27" xr3:uid="{72913F84-BFE6-4F18-B568-78A034CF91E0}" name="Serie mouse" dataDxfId="57"/>
+    <tableColumn id="28" xr3:uid="{9503ECC5-F543-47DD-B05F-BE5CFED614E7}" name="Inventario CPU" dataDxfId="56"/>
+    <tableColumn id="29" xr3:uid="{F23D81CF-45FF-4B42-AE1D-C3FF20A02D47}" name="Inventario Monitor" dataDxfId="55"/>
+    <tableColumn id="30" xr3:uid="{5E7F41A6-23EE-49FF-B9A7-67B41746BA02}" name="Inventario Teclado" dataDxfId="54"/>
+    <tableColumn id="31" xr3:uid="{E73A3977-4E78-4BBD-B43C-5CDDDFB5A0B5}" name="Inventario Mouse" dataDxfId="53"/>
     <tableColumn id="32" xr3:uid="{132BAE04-41F0-4D14-886F-EE4B5E17AA48}" name="Observación"/>
-    <tableColumn id="33" xr3:uid="{75F5651F-591E-4487-8692-3B6B587F55ED}" name="Fecha si se hace cambio"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{65571BBC-6721-44F4-B921-CE5855D2DD45}" name="Tabla13" displayName="Tabla13" ref="A1:L2" insertRow="1" totalsRowShown="0" headerRowDxfId="49" dataDxfId="47" headerRowBorderDxfId="48" tableBorderDxfId="46">
-  <autoFilter ref="A1:L2" xr:uid="{65571BBC-6721-44F4-B921-CE5855D2DD45}"/>
-  <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{FDE9EEEE-D60D-45CB-A800-B53803E8A3B8}" name="N°" dataDxfId="45"/>
-    <tableColumn id="9" xr3:uid="{0F2C1BC4-B276-43C3-8519-94D5DE11E4D7}" name="Año Adq" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{1B2D9558-F9ED-4CCE-9E02-C266643535C2}" name="Inventario" dataDxfId="44"/>
-    <tableColumn id="4" xr3:uid="{F9374C12-7D10-4F8D-A9F2-6B74A4324A16}" name="Bloque" dataDxfId="43"/>
-    <tableColumn id="5" xr3:uid="{CC47AE73-F008-4779-8A1E-999613B73F36}" name="Ubicación" dataDxfId="42"/>
-    <tableColumn id="6" xr3:uid="{C4B7087C-C5A9-418F-973B-91019B7B4D85}" name="Marca" dataDxfId="41"/>
-    <tableColumn id="7" xr3:uid="{A29FE592-5D13-4856-A8B2-D3757F7FE5D1}" name="Modelo" dataDxfId="40"/>
-    <tableColumn id="35" xr3:uid="{28CE02F8-C218-4318-91D6-3221A4C1677C}" name="Serie" dataDxfId="39"/>
-    <tableColumn id="8" xr3:uid="{D6339E67-64E9-4609-AE94-03511A1E2DFA}" name="Categoría" dataDxfId="38"/>
-    <tableColumn id="10" xr3:uid="{BC81D9A6-A156-4735-B029-2F2D63CB0EBE}" name="Lámpara" dataDxfId="37"/>
-    <tableColumn id="11" xr3:uid="{EC220C64-81F8-4715-812E-830F143FAFE1}" name="Estado" dataDxfId="36"/>
-    <tableColumn id="12" xr3:uid="{520BC8C9-05B0-4EE0-A833-D9F61A0DD0AB}" name="Observación" dataDxfId="35"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{65571BBC-6721-44F4-B921-CE5855D2DD45}" name="Tabla13" displayName="Tabla13" ref="A1:M2" insertRow="1" totalsRowShown="0" headerRowDxfId="52" dataDxfId="50" headerRowBorderDxfId="51" tableBorderDxfId="49">
+  <autoFilter ref="A1:M2" xr:uid="{65571BBC-6721-44F4-B921-CE5855D2DD45}"/>
+  <tableColumns count="13">
+    <tableColumn id="1" xr3:uid="{FDE9EEEE-D60D-45CB-A800-B53803E8A3B8}" name="N°" dataDxfId="48"/>
+    <tableColumn id="9" xr3:uid="{0F2C1BC4-B276-43C3-8519-94D5DE11E4D7}" name="Año Adq" dataDxfId="47"/>
+    <tableColumn id="2" xr3:uid="{0C5F1C16-6E4F-4314-9E46-938258FF3548}" name="Empresa" dataDxfId="46"/>
+    <tableColumn id="3" xr3:uid="{1B2D9558-F9ED-4CCE-9E02-C266643535C2}" name="Inventario" dataDxfId="45"/>
+    <tableColumn id="4" xr3:uid="{F9374C12-7D10-4F8D-A9F2-6B74A4324A16}" name="Bloque" dataDxfId="44"/>
+    <tableColumn id="5" xr3:uid="{CC47AE73-F008-4779-8A1E-999613B73F36}" name="Ubicación" dataDxfId="43"/>
+    <tableColumn id="6" xr3:uid="{C4B7087C-C5A9-418F-973B-91019B7B4D85}" name="Marca" dataDxfId="42"/>
+    <tableColumn id="7" xr3:uid="{A29FE592-5D13-4856-A8B2-D3757F7FE5D1}" name="Modelo" dataDxfId="41"/>
+    <tableColumn id="35" xr3:uid="{28CE02F8-C218-4318-91D6-3221A4C1677C}" name="Serie" dataDxfId="40"/>
+    <tableColumn id="8" xr3:uid="{D6339E67-64E9-4609-AE94-03511A1E2DFA}" name="Categoría" dataDxfId="39"/>
+    <tableColumn id="10" xr3:uid="{BC81D9A6-A156-4735-B029-2F2D63CB0EBE}" name="Lámpara" dataDxfId="38"/>
+    <tableColumn id="11" xr3:uid="{EC220C64-81F8-4715-812E-830F143FAFE1}" name="Estado" dataDxfId="37"/>
+    <tableColumn id="12" xr3:uid="{520BC8C9-05B0-4EE0-A833-D9F61A0DD0AB}" name="Observación" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{117726C3-B927-45D2-BCB6-906E81362D65}" name="Tabla134" displayName="Tabla134" ref="A1:L2" insertRow="1" totalsRowShown="0" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33" tableBorderDxfId="31">
-  <autoFilter ref="A1:L2" xr:uid="{117726C3-B927-45D2-BCB6-906E81362D65}"/>
-  <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{276C8004-7E62-4A99-99B6-54C1CCAB9A0D}" name="N°" dataDxfId="30"/>
-    <tableColumn id="8" xr3:uid="{5DC544D0-D6BC-4180-8835-12C885A89DB4}" name="Año Adq" dataDxfId="1"/>
-    <tableColumn id="59" xr3:uid="{2EDF8951-57A8-4DA8-83DD-41E4ABB04F28}" name="Nombre" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{6C6FAF5E-4416-4701-AF7F-C6B09875F0E3}" name="Inventario" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{9009A994-0659-4EB2-A948-BB850B7E7869}" name="Bloque" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{2BFE8A4C-F74C-4478-94F2-9CDCD7517FF5}" name="Ubicación" dataDxfId="26"/>
-    <tableColumn id="6" xr3:uid="{C3F80FC4-FC88-4067-86B5-9E0F39992776}" name="Marca" dataDxfId="25"/>
-    <tableColumn id="7" xr3:uid="{1EB67BDD-CF6B-448D-A8ED-A99A60F26085}" name="Modelo" dataDxfId="24"/>
-    <tableColumn id="35" xr3:uid="{4F1E28EC-460F-4A15-A541-75DDC5A3B10F}" name="Serie" dataDxfId="23"/>
-    <tableColumn id="11" xr3:uid="{646DF198-108C-4FD8-BA3F-221C547C787D}" name="MAC" dataDxfId="22"/>
-    <tableColumn id="61" xr3:uid="{0F76C99C-FD25-4F18-AC82-BC0A9BD0BFC3}" name="Estado" dataDxfId="21"/>
-    <tableColumn id="12" xr3:uid="{DA153594-3249-41ED-9088-5D447B2330F5}" name="Observación" dataDxfId="20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{117726C3-B927-45D2-BCB6-906E81362D65}" name="Tabla134" displayName="Tabla134" ref="A1:M2" insertRow="1" totalsRowShown="0" headerRowDxfId="35" dataDxfId="33" headerRowBorderDxfId="34" tableBorderDxfId="32">
+  <autoFilter ref="A1:M2" xr:uid="{117726C3-B927-45D2-BCB6-906E81362D65}"/>
+  <tableColumns count="13">
+    <tableColumn id="1" xr3:uid="{276C8004-7E62-4A99-99B6-54C1CCAB9A0D}" name="N°" dataDxfId="31"/>
+    <tableColumn id="8" xr3:uid="{5DC544D0-D6BC-4180-8835-12C885A89DB4}" name="Año Adq" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{AA105BF1-5DE3-460B-BF8F-1DECA17B41EE}" name="Empresa" dataDxfId="29"/>
+    <tableColumn id="59" xr3:uid="{2EDF8951-57A8-4DA8-83DD-41E4ABB04F28}" name="Nombre" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{6C6FAF5E-4416-4701-AF7F-C6B09875F0E3}" name="Inventario" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{9009A994-0659-4EB2-A948-BB850B7E7869}" name="Bloque" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{2BFE8A4C-F74C-4478-94F2-9CDCD7517FF5}" name="Ubicación" dataDxfId="25"/>
+    <tableColumn id="6" xr3:uid="{C3F80FC4-FC88-4067-86B5-9E0F39992776}" name="Marca" dataDxfId="24"/>
+    <tableColumn id="7" xr3:uid="{1EB67BDD-CF6B-448D-A8ED-A99A60F26085}" name="Modelo" dataDxfId="23"/>
+    <tableColumn id="35" xr3:uid="{4F1E28EC-460F-4A15-A541-75DDC5A3B10F}" name="Serie" dataDxfId="22"/>
+    <tableColumn id="11" xr3:uid="{646DF198-108C-4FD8-BA3F-221C547C787D}" name="MAC" dataDxfId="21"/>
+    <tableColumn id="61" xr3:uid="{0F76C99C-FD25-4F18-AC82-BC0A9BD0BFC3}" name="Estado" dataDxfId="20"/>
+    <tableColumn id="12" xr3:uid="{DA153594-3249-41ED-9088-5D447B2330F5}" name="Observación" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{81C6E5BE-3A2E-49E1-B3C1-BD159715F86B}" name="Tabla1345" displayName="Tabla1345" ref="A1:N2" insertRow="1" totalsRowShown="0" headerRowDxfId="19" dataDxfId="17" headerRowBorderDxfId="18" tableBorderDxfId="16">
-  <autoFilter ref="A1:N2" xr:uid="{81C6E5BE-3A2E-49E1-B3C1-BD159715F86B}"/>
-  <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{5752E7FC-405F-447F-B9C8-E1DD962FB1D1}" name="N°" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{8DECD9A9-F47F-4F5A-B630-9B1F78EDD65B}" name="Año Adq" dataDxfId="0"/>
-    <tableColumn id="59" xr3:uid="{6E508FCA-0F19-4A5A-97A2-4220449D6882}" name="Nombre" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{F0B5BEAE-2A98-4302-9893-9D181D3E666D}" name="Inventario" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{1F479286-0DEA-4626-AB22-A4F8CC3FE875}" name="Bloque" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{93646E9B-68FE-417A-98DE-28980ED118D4}" name="Ubicación" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{D153A63A-4284-4B63-AC79-C4EAB8A15D1F}" name="Marca" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{C69FBE1A-5E88-4580-8C50-3D16B56FC37D}" name="Modelo" dataDxfId="9"/>
-    <tableColumn id="35" xr3:uid="{669AFF80-A616-4FFA-BA41-D36E9D103A74}" name="Serie" dataDxfId="8"/>
-    <tableColumn id="11" xr3:uid="{D3822BF8-4C38-4CBA-A4FB-906635BE0D3C}" name="MAC" dataDxfId="7"/>
-    <tableColumn id="62" xr3:uid="{2FB33EDF-D0A6-4D55-9A71-7AFA57C20872}" name="Puertos" dataDxfId="6"/>
-    <tableColumn id="63" xr3:uid="{B25EF247-15A5-4E8D-86D3-C87008833029}" name="Puertos FTP" dataDxfId="5"/>
-    <tableColumn id="61" xr3:uid="{25955EE6-0956-42D8-B04D-AA175B1FCD83}" name="Estado" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{1CBC6A15-3C59-4C4B-8DDC-87EA4A40B0E6}" name="Observación" dataDxfId="3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{81C6E5BE-3A2E-49E1-B3C1-BD159715F86B}" name="Tabla1345" displayName="Tabla1345" ref="A1:O2" insertRow="1" totalsRowShown="0" headerRowDxfId="18" dataDxfId="16" headerRowBorderDxfId="17" tableBorderDxfId="15">
+  <autoFilter ref="A1:O2" xr:uid="{81C6E5BE-3A2E-49E1-B3C1-BD159715F86B}"/>
+  <tableColumns count="15">
+    <tableColumn id="1" xr3:uid="{5752E7FC-405F-447F-B9C8-E1DD962FB1D1}" name="N°" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{8DECD9A9-F47F-4F5A-B630-9B1F78EDD65B}" name="Año Adq" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{1025115D-C0E7-40B8-8800-C25D234509A0}" name="Empresa" dataDxfId="12"/>
+    <tableColumn id="59" xr3:uid="{6E508FCA-0F19-4A5A-97A2-4220449D6882}" name="Nombre" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{F0B5BEAE-2A98-4302-9893-9D181D3E666D}" name="Inventario" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{1F479286-0DEA-4626-AB22-A4F8CC3FE875}" name="Bloque" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{93646E9B-68FE-417A-98DE-28980ED118D4}" name="Ubicación" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{D153A63A-4284-4B63-AC79-C4EAB8A15D1F}" name="Marca" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{C69FBE1A-5E88-4580-8C50-3D16B56FC37D}" name="Modelo" dataDxfId="6"/>
+    <tableColumn id="35" xr3:uid="{669AFF80-A616-4FFA-BA41-D36E9D103A74}" name="Serie" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{D3822BF8-4C38-4CBA-A4FB-906635BE0D3C}" name="MAC" dataDxfId="4"/>
+    <tableColumn id="62" xr3:uid="{2FB33EDF-D0A6-4D55-9A71-7AFA57C20872}" name="Puertos" dataDxfId="3"/>
+    <tableColumn id="63" xr3:uid="{B25EF247-15A5-4E8D-86D3-C87008833029}" name="Puertos FTP" dataDxfId="2"/>
+    <tableColumn id="61" xr3:uid="{25955EE6-0956-42D8-B04D-AA175B1FCD83}" name="Estado" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{1CBC6A15-3C59-4C4B-8DDC-87EA4A40B0E6}" name="Observación" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1282,32 +1313,32 @@
     <col min="5" max="5" width="28.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.85546875" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="19.42578125" customWidth="1"/>
-    <col min="14" max="14" width="13" customWidth="1"/>
-    <col min="15" max="15" width="20.5703125" customWidth="1"/>
-    <col min="16" max="17" width="16.42578125" customWidth="1"/>
-    <col min="18" max="18" width="13" style="4" customWidth="1"/>
-    <col min="19" max="19" width="14.5703125" style="4" customWidth="1"/>
-    <col min="20" max="20" width="11.7109375" style="5" customWidth="1"/>
-    <col min="21" max="21" width="16" style="4" customWidth="1"/>
-    <col min="22" max="22" width="17.5703125" style="4" customWidth="1"/>
-    <col min="23" max="23" width="15.28515625" style="5" customWidth="1"/>
-    <col min="24" max="24" width="15.42578125" style="4" customWidth="1"/>
-    <col min="25" max="25" width="17" style="4" customWidth="1"/>
-    <col min="26" max="26" width="14.7109375" style="5" customWidth="1"/>
-    <col min="27" max="27" width="14.85546875" style="4" customWidth="1"/>
-    <col min="28" max="28" width="16.42578125" style="4" customWidth="1"/>
-    <col min="29" max="29" width="14.140625" style="5" customWidth="1"/>
-    <col min="30" max="30" width="16.28515625" style="4" customWidth="1"/>
-    <col min="31" max="31" width="19.85546875" style="4" customWidth="1"/>
-    <col min="32" max="32" width="19.5703125" style="4" customWidth="1"/>
-    <col min="33" max="33" width="18.7109375" style="4" customWidth="1"/>
-    <col min="34" max="34" width="14.140625" customWidth="1"/>
-    <col min="35" max="35" width="24" customWidth="1"/>
+    <col min="8" max="8" width="10.28515625" customWidth="1"/>
+    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.85546875" customWidth="1"/>
+    <col min="12" max="12" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="19.42578125" customWidth="1"/>
+    <col min="15" max="15" width="13" customWidth="1"/>
+    <col min="16" max="16" width="20.5703125" customWidth="1"/>
+    <col min="17" max="18" width="16.42578125" customWidth="1"/>
+    <col min="19" max="19" width="13" style="4" customWidth="1"/>
+    <col min="20" max="20" width="14.5703125" style="4" customWidth="1"/>
+    <col min="21" max="21" width="11.7109375" style="5" customWidth="1"/>
+    <col min="22" max="22" width="16" style="4" customWidth="1"/>
+    <col min="23" max="23" width="17.5703125" style="4" customWidth="1"/>
+    <col min="24" max="24" width="15.28515625" style="5" customWidth="1"/>
+    <col min="25" max="25" width="15.42578125" style="4" customWidth="1"/>
+    <col min="26" max="26" width="17" style="4" customWidth="1"/>
+    <col min="27" max="27" width="14.7109375" style="5" customWidth="1"/>
+    <col min="28" max="28" width="14.85546875" style="4" customWidth="1"/>
+    <col min="29" max="29" width="16.42578125" style="4" customWidth="1"/>
+    <col min="30" max="30" width="14.140625" style="5" customWidth="1"/>
+    <col min="31" max="31" width="16.28515625" style="4" customWidth="1"/>
+    <col min="32" max="32" width="19.85546875" style="4" customWidth="1"/>
+    <col min="33" max="33" width="19.5703125" style="4" customWidth="1"/>
+    <col min="34" max="34" width="18.7109375" style="4" customWidth="1"/>
+    <col min="35" max="35" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
@@ -1332,89 +1363,89 @@
       <c r="G1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="I1" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="AA1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AD1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.25">
@@ -1432,6 +1463,7 @@
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1443,21 +1475,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEBB0042-A0FD-49A0-A2B5-EF98DD6502FD}">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="12" max="12" width="38.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>41</v>
@@ -1468,163 +1500,29 @@
       <c r="F1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="I1" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="J1" s="1" t="s">
+      <c r="I1" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>47</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED870B1E-1F89-4BB2-9D46-7F5FA05B9BFD}">
-  <dimension ref="A1:L2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="I1" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E7B876E-210B-4FAF-A1A3-6F9B8A1F3B53}">
-  <dimension ref="A1:N2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="I1" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>33</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>46</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="N1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="6"/>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -1638,7 +1536,6 @@
       <c r="K2" s="7"/>
       <c r="L2" s="7"/>
       <c r="M2" s="7"/>
-      <c r="N2" s="7"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1647,4 +1544,152 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED870B1E-1F89-4BB2-9D46-7F5FA05B9BFD}">
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="6"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E7B876E-210B-4FAF-A1A3-6F9B8A1F3B53}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="6"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>